<commit_message>
SABBB KUCHHH HAI BHAIII
</commit_message>
<xml_diff>
--- a/data/daily/attendance.xlsx
+++ b/data/daily/attendance.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="207">
   <si>
     <t>Total</t>
   </si>
@@ -22,16 +22,22 @@
     <t>Username</t>
   </si>
   <si>
-    <t>Apr 20, 2026</t>
+    <t>Apr 25, 2026</t>
+  </si>
+  <si>
+    <t>Dillip Kumar Mohanty</t>
+  </si>
+  <si>
+    <t>dillip_st</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
   <si>
     <t>Pranjal Gupta</t>
   </si>
   <si>
     <t>pranjal_st</t>
-  </si>
-  <si>
-    <t>A</t>
   </si>
   <si>
     <t>Vaibhav Prabhakar Kamble</t>
@@ -1038,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="20"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1085,7 +1091,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
@@ -1094,21 +1100,21 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1127,7 +1133,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>16</v>
@@ -1136,12 +1142,12 @@
         <v>17</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>18</v>
@@ -1150,7 +1156,7 @@
         <v>19</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1248,12 +1254,12 @@
         <v>33</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>34</v>
@@ -1262,12 +1268,12 @@
         <v>35</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>36</v>
@@ -1276,12 +1282,12 @@
         <v>37</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>38</v>
@@ -1290,7 +1296,7 @@
         <v>39</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1309,7 +1315,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>42</v>
@@ -1318,7 +1324,7 @@
         <v>43</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1332,12 +1338,12 @@
         <v>45</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>46</v>
@@ -1346,7 +1352,7 @@
         <v>47</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1379,7 +1385,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>52</v>
@@ -1388,7 +1394,7 @@
         <v>53</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1402,7 +1408,7 @@
         <v>55</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1416,12 +1422,12 @@
         <v>57</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>58</v>
@@ -1430,7 +1436,7 @@
         <v>59</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1444,7 +1450,7 @@
         <v>61</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1458,12 +1464,12 @@
         <v>63</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>64</v>
@@ -1472,12 +1478,12 @@
         <v>65</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>66</v>
@@ -1486,7 +1492,7 @@
         <v>67</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1500,7 +1506,7 @@
         <v>69</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1514,7 +1520,7 @@
         <v>71</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1528,12 +1534,12 @@
         <v>73</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>74</v>
@@ -1542,12 +1548,12 @@
         <v>75</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>76</v>
@@ -1556,7 +1562,7 @@
         <v>77</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1570,7 +1576,7 @@
         <v>79</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1584,7 +1590,7 @@
         <v>81</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1598,7 +1604,7 @@
         <v>83</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1612,7 +1618,7 @@
         <v>85</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1626,12 +1632,12 @@
         <v>87</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>88</v>
@@ -1640,7 +1646,7 @@
         <v>89</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1654,12 +1660,12 @@
         <v>91</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>92</v>
@@ -1668,7 +1674,7 @@
         <v>93</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1682,7 +1688,7 @@
         <v>95</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1696,7 +1702,7 @@
         <v>97</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1710,7 +1716,7 @@
         <v>99</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1724,7 +1730,7 @@
         <v>101</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1738,7 +1744,7 @@
         <v>103</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1752,7 +1758,7 @@
         <v>105</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1766,7 +1772,7 @@
         <v>107</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -1780,7 +1786,7 @@
         <v>109</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -1794,12 +1800,12 @@
         <v>111</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>112</v>
@@ -1808,12 +1814,12 @@
         <v>113</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>114</v>
@@ -1822,12 +1828,12 @@
         <v>115</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>116</v>
@@ -1836,12 +1842,12 @@
         <v>117</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>118</v>
@@ -1850,7 +1856,7 @@
         <v>119</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -1864,7 +1870,7 @@
         <v>121</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -1878,7 +1884,7 @@
         <v>123</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -1892,7 +1898,7 @@
         <v>125</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -1906,7 +1912,7 @@
         <v>127</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -1920,7 +1926,7 @@
         <v>129</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -1934,12 +1940,12 @@
         <v>131</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>132</v>
@@ -1948,12 +1954,12 @@
         <v>133</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>134</v>
@@ -1962,7 +1968,7 @@
         <v>135</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -1976,7 +1982,7 @@
         <v>137</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -1990,12 +1996,12 @@
         <v>139</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>140</v>
@@ -2004,7 +2010,7 @@
         <v>141</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2449,9 +2455,23 @@
         <v>204</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D101" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="2">
+        <v>0</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D102" s="2" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>